<commit_message>
fix(beasiswa): resolve TDZ runtime crash caused by pUPActive declaration order
</commit_message>
<xml_diff>
--- a/Data_Monitoring_PPDB_AlImam_Final_V8.xlsx
+++ b/Data_Monitoring_PPDB_AlImam_Final_V8.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40635EF5-F354-4E6F-AEDD-35647640738E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD86EE7F-9372-4F1A-9D87-6024BEA7324C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="308">
   <si>
     <t>DATA MONITORING PPDB MTs - AL ANDALUS AL IMAM</t>
   </si>
@@ -74,9 +74,6 @@
     <t>7371111406140004</t>
   </si>
   <si>
-    <t>ATQANUL UMMAH AHMAD</t>
-  </si>
-  <si>
     <t>MTs</t>
   </si>
   <si>
@@ -314,9 +311,6 @@
     <t>3173081608131003</t>
   </si>
   <si>
-    <t>MUHAMMAD RIFQI HAMID</t>
-  </si>
-  <si>
     <t>SDN Meruya Utara 10 Pagi</t>
   </si>
   <si>
@@ -425,9 +419,6 @@
     <t>3174080703141001</t>
   </si>
   <si>
-    <t>muhammad Azzam Al hafiz</t>
-  </si>
-  <si>
     <t>MI Saadatudarain</t>
   </si>
   <si>
@@ -485,9 +476,6 @@
     <t>Daffa Muammar Dzaki</t>
   </si>
   <si>
-    <t>SMPIT IHYA AS-SUNNAH TASIKMALAYA</t>
-  </si>
-  <si>
     <t>Samsul Aripin</t>
   </si>
   <si>
@@ -503,12 +491,6 @@
     <t>3172011210101003</t>
   </si>
   <si>
-    <t>FARID</t>
-  </si>
-  <si>
-    <t>AN NAJAH</t>
-  </si>
-  <si>
     <t>Fauzan</t>
   </si>
   <si>
@@ -524,12 +506,6 @@
     <t>3201132910100005</t>
   </si>
   <si>
-    <t>FAVIAN RADI</t>
-  </si>
-  <si>
-    <t>RAUDHATUL MUHIBBIN</t>
-  </si>
-  <si>
     <t>Abdul Ismail</t>
   </si>
   <si>
@@ -599,9 +575,6 @@
     <t>3175071007111003</t>
   </si>
   <si>
-    <t>KHUBAIB ABDUL AZIZ</t>
-  </si>
-  <si>
     <t>Pondok Pesantren Ibnu Abbas</t>
   </si>
   <si>
@@ -623,9 +596,6 @@
     <t>Ken Alfarezha Haryadi</t>
   </si>
   <si>
-    <t>MTA AT Tauhid Pangkalpinang</t>
-  </si>
-  <si>
     <t>Haryadi</t>
   </si>
   <si>
@@ -641,12 +611,6 @@
     <t>5202011801110001</t>
   </si>
   <si>
-    <t>LALU MUHAMAD RIZKY ANANDA</t>
-  </si>
-  <si>
-    <t>PKBM ARRISALAH LOMBOK</t>
-  </si>
-  <si>
     <t>LALU USMAN ALI</t>
   </si>
   <si>
@@ -665,9 +629,6 @@
     <t>Miizan Alghifary Dizlilar</t>
   </si>
   <si>
-    <t>SMP tahfidz alfitrah 2</t>
-  </si>
-  <si>
     <t>Asep mulyadi</t>
   </si>
   <si>
@@ -686,9 +647,6 @@
     <t>Muhammad Hafidz Abdurrahman</t>
   </si>
   <si>
-    <t>Pesantren Tahfidz Al Islah</t>
-  </si>
-  <si>
     <t>Chairul Tirta</t>
   </si>
   <si>
@@ -707,9 +665,6 @@
     <t>Muhammad Khoirul Azzam</t>
   </si>
   <si>
-    <t>Pondok pesantren AL-ISLAH</t>
-  </si>
-  <si>
     <t>Siti Mahzuroh</t>
   </si>
   <si>
@@ -791,9 +746,6 @@
     <t>Raylan Akbar</t>
   </si>
   <si>
-    <t>SMPIT AL INSAN TAUHUD SCHOOL</t>
-  </si>
-  <si>
     <t>Agus Supendi</t>
   </si>
   <si>
@@ -900,6 +852,99 @@
   </si>
   <si>
     <t>PKBM Bangun Bangsa</t>
+  </si>
+  <si>
+    <t>MTsN 3 Lembata</t>
+  </si>
+  <si>
+    <t>Bapa Rahmat</t>
+  </si>
+  <si>
+    <t>Intan Abdullah</t>
+  </si>
+  <si>
+    <t>Ratna Sari Ningsih</t>
+  </si>
+  <si>
+    <t>PKBM KT-IPMA</t>
+  </si>
+  <si>
+    <t>Cecep Dhian Rusdiana</t>
+  </si>
+  <si>
+    <t>Atin Supriatin</t>
+  </si>
+  <si>
+    <t>Andrian Arisandy Siagian</t>
+  </si>
+  <si>
+    <t>Nurul Syarifah</t>
+  </si>
+  <si>
+    <t>Mustangin</t>
+  </si>
+  <si>
+    <t>Wati Melasari</t>
+  </si>
+  <si>
+    <t>PKBM Al Andalus</t>
+  </si>
+  <si>
+    <t>Heriyanto</t>
+  </si>
+  <si>
+    <t>Novy</t>
+  </si>
+  <si>
+    <t>PKBM Wijaya Kusuma</t>
+  </si>
+  <si>
+    <t>Pondok Pesantren Al-Ishlah</t>
+  </si>
+  <si>
+    <t>SMPIT Al Insan Tauhud School</t>
+  </si>
+  <si>
+    <t>Pesantren Tahfidz Al-Ishlah</t>
+  </si>
+  <si>
+    <t>SMP Tahfidz Alfitrah 2</t>
+  </si>
+  <si>
+    <t>PKBM Ar-Risalah Lombok</t>
+  </si>
+  <si>
+    <t>MTA AT Tauhid Pangkal Pinang</t>
+  </si>
+  <si>
+    <t>Raudhatul Muhibbin</t>
+  </si>
+  <si>
+    <t>An-Najah</t>
+  </si>
+  <si>
+    <t>SMPIT Ihya As-Sunnah Tasikmalaya</t>
+  </si>
+  <si>
+    <t>Farid</t>
+  </si>
+  <si>
+    <t>Favian Radi</t>
+  </si>
+  <si>
+    <t>Khubaib Abdul Aziz</t>
+  </si>
+  <si>
+    <t>Lalu Muhamad Rizky Ananda</t>
+  </si>
+  <si>
+    <t>Atqanul Ummah Ahmad</t>
+  </si>
+  <si>
+    <t>Muhammad Rifqi Hamid</t>
+  </si>
+  <si>
+    <t>Muhammad Azzam Al Hafiz</t>
   </si>
 </sst>
 </file>
@@ -1410,37 +1455,37 @@
         <v>16</v>
       </c>
       <c r="D4" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>18</v>
-      </c>
       <c r="F4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G4" s="3" t="s">
-        <v>20</v>
-      </c>
       <c r="H4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I4" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="J4" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="K4" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="K4" s="3" t="s">
-        <v>24</v>
-      </c>
       <c r="L4" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>275</v>
+        <v>259</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.35">
@@ -1448,43 +1493,43 @@
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G5" s="3" t="s">
+      <c r="H5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I5" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="H5" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I5" s="3" t="s">
+      <c r="J5" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="J5" s="3" t="s">
+      <c r="K5" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="K5" s="3" t="s">
-        <v>34</v>
-      </c>
       <c r="L5" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.35">
@@ -1492,43 +1537,43 @@
         <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="E6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>292</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I6" s="3" t="s">
+      <c r="J6" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="J6" s="3" t="s">
+      <c r="K6" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="K6" s="3" t="s">
-        <v>40</v>
-      </c>
       <c r="L6" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>275</v>
+        <v>259</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.35">
@@ -1536,43 +1581,43 @@
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="E7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I7" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>291</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I7" s="3" t="s">
+      <c r="J7" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="J7" s="3" t="s">
+      <c r="K7" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="K7" s="3" t="s">
-        <v>46</v>
-      </c>
       <c r="L7" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>275</v>
+        <v>259</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.35">
@@ -1580,43 +1625,43 @@
         <v>5</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="E8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I8" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>290</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I8" s="3" t="s">
+      <c r="J8" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="J8" s="3" t="s">
+      <c r="K8" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="K8" s="3" t="s">
-        <v>52</v>
-      </c>
       <c r="L8" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>275</v>
+        <v>259</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.35">
@@ -1624,43 +1669,43 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="E9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G9" s="3" t="s">
+      <c r="H9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I9" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="H9" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I9" s="3" t="s">
+      <c r="J9" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="J9" s="3" t="s">
+      <c r="K9" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="K9" s="3" t="s">
-        <v>59</v>
-      </c>
       <c r="L9" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
@@ -1668,43 +1713,43 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="E10" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G10" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G10" s="3" t="s">
+      <c r="H10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I10" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="H10" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I10" s="3" t="s">
+      <c r="J10" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="J10" s="3" t="s">
+      <c r="K10" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="K10" s="3" t="s">
-        <v>66</v>
-      </c>
       <c r="L10" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.35">
@@ -1712,43 +1757,43 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="E11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G11" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G11" s="3" t="s">
+      <c r="H11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I11" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="H11" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I11" s="3" t="s">
+      <c r="J11" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="J11" s="3" t="s">
+      <c r="K11" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="K11" s="3" t="s">
-        <v>73</v>
-      </c>
       <c r="L11" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.35">
@@ -1756,43 +1801,43 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="E12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="K12" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="E12" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>277</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I12" s="3" t="s">
-        <v>279</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>286</v>
-      </c>
-      <c r="K12" s="3" t="s">
-        <v>77</v>
-      </c>
       <c r="L12" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.35">
@@ -1800,43 +1845,43 @@
         <v>10</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="D13" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="E13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I13" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="E13" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I13" s="3" t="s">
+      <c r="J13" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="J13" s="3" t="s">
+      <c r="K13" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="K13" s="3" t="s">
-        <v>83</v>
-      </c>
       <c r="L13" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.35">
@@ -1844,43 +1889,43 @@
         <v>11</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="E14" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G14" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="E14" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G14" s="3" t="s">
+      <c r="H14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I14" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="H14" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I14" s="3" t="s">
+      <c r="J14" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="J14" s="3" t="s">
+      <c r="K14" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="K14" s="3" t="s">
-        <v>90</v>
-      </c>
       <c r="L14" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.35">
@@ -1888,43 +1933,43 @@
         <v>12</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="E15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="K15" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="E15" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>278</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I15" s="3" t="s">
-        <v>280</v>
-      </c>
-      <c r="J15" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="K15" s="3" t="s">
-        <v>94</v>
-      </c>
       <c r="L15" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M15" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="M15" s="2" t="s">
-        <v>26</v>
-      </c>
       <c r="N15" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.35">
@@ -1932,43 +1977,43 @@
         <v>13</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="D16" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G16" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="H16" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="K16" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="E16" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I16" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="J16" s="3" t="s">
-        <v>282</v>
-      </c>
-      <c r="K16" s="3" t="s">
-        <v>99</v>
-      </c>
       <c r="L16" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>275</v>
+        <v>259</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.35">
@@ -1976,43 +2021,43 @@
         <v>14</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D17" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="E17" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I17" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="J17" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="E17" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I17" s="3" t="s">
+      <c r="K17" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="J17" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="K17" s="3" t="s">
-        <v>105</v>
-      </c>
       <c r="L17" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.35">
@@ -2020,43 +2065,43 @@
         <v>15</v>
       </c>
       <c r="B18" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D18" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="E18" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G18" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="H18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I18" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="E18" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G18" s="3" t="s">
+      <c r="J18" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="K18" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="H18" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="J18" s="3" t="s">
-        <v>283</v>
-      </c>
-      <c r="K18" s="3" t="s">
-        <v>111</v>
-      </c>
       <c r="L18" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>275</v>
+        <v>259</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.35">
@@ -2064,43 +2109,43 @@
         <v>16</v>
       </c>
       <c r="B19" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D19" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="E19" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G19" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="H19" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I19" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="E19" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G19" s="3" t="s">
+      <c r="J19" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="H19" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I19" s="3" t="s">
+      <c r="K19" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="J19" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="K19" s="3" t="s">
-        <v>118</v>
-      </c>
       <c r="L19" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>275</v>
+        <v>259</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.35">
@@ -2108,43 +2153,43 @@
         <v>17</v>
       </c>
       <c r="B20" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="D20" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="E20" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G20" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="H20" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I20" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="E20" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G20" s="3" t="s">
+      <c r="J20" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="H20" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I20" s="3" t="s">
+      <c r="K20" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="J20" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="K20" s="3" t="s">
-        <v>125</v>
-      </c>
       <c r="L20" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.35">
@@ -2152,43 +2197,43 @@
         <v>18</v>
       </c>
       <c r="B21" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D21" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="E21" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I21" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="J21" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="E21" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G21" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I21" s="3" t="s">
+      <c r="K21" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="J21" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="K21" s="3" t="s">
-        <v>131</v>
-      </c>
       <c r="L21" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M21" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="M21" s="2" t="s">
-        <v>26</v>
-      </c>
       <c r="N21" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.35">
@@ -2196,43 +2241,43 @@
         <v>19</v>
       </c>
       <c r="B22" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G22" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="H22" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I22" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="J22" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="K22" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="E22" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G22" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I22" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="J22" s="3" t="s">
-        <v>284</v>
-      </c>
-      <c r="K22" s="3" t="s">
-        <v>137</v>
-      </c>
       <c r="L22" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>275</v>
+        <v>259</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -2263,7 +2308,7 @@
     <col min="4" max="4" width="35" customWidth="1"/>
     <col min="5" max="5" width="10" customWidth="1"/>
     <col min="6" max="6" width="15" customWidth="1"/>
-    <col min="7" max="7" width="30" customWidth="1"/>
+    <col min="7" max="7" width="53" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
     <col min="9" max="10" width="25" customWidth="1"/>
     <col min="11" max="11" width="20" customWidth="1"/>
@@ -2274,7 +2319,7 @@
   <sheetData>
     <row r="1" spans="1:14" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -2339,43 +2384,43 @@
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="F4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="K4" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>143</v>
-      </c>
       <c r="L4" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.35">
@@ -2383,43 +2428,43 @@
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="H5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I5" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="J5" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G5" s="3" t="s">
+      <c r="K5" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="H5" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>150</v>
-      </c>
       <c r="L5" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.35">
@@ -2427,43 +2472,43 @@
         <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="J6" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="K6" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="J6" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="K6" s="3" t="s">
-        <v>157</v>
-      </c>
       <c r="L6" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.35">
@@ -2471,43 +2516,43 @@
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="K7" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="K7" s="3" t="s">
-        <v>164</v>
-      </c>
       <c r="L7" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.35">
@@ -2515,43 +2560,43 @@
         <v>5</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>167</v>
+        <v>302</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>168</v>
+        <v>298</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>275</v>
+        <v>259</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.35">
@@ -2559,43 +2604,43 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="L9" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M9" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="M9" s="2" t="s">
-        <v>26</v>
-      </c>
       <c r="N9" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
@@ -2603,43 +2648,41 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>32</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="G10" s="3"/>
       <c r="H10" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>32</v>
+        <v>280</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.35">
@@ -2647,43 +2690,43 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.35">
@@ -2691,43 +2734,43 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>192</v>
+        <v>303</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>195</v>
+        <v>186</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>196</v>
+        <v>187</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>275</v>
+        <v>259</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.35">
@@ -2735,43 +2778,43 @@
         <v>10</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>197</v>
+        <v>188</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>199</v>
+        <v>190</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>200</v>
+        <v>297</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>203</v>
+        <v>193</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.35">
@@ -2779,43 +2822,43 @@
         <v>11</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>206</v>
+        <v>304</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>207</v>
+        <v>296</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.35">
@@ -2823,43 +2866,43 @@
         <v>12</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>211</v>
+        <v>199</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>214</v>
+        <v>295</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>215</v>
+        <v>202</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>216</v>
+        <v>203</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>217</v>
+        <v>204</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.35">
@@ -2867,43 +2910,43 @@
         <v>13</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>218</v>
+        <v>205</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>219</v>
+        <v>206</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>220</v>
+        <v>207</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>221</v>
+        <v>294</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>222</v>
+        <v>208</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>223</v>
+        <v>209</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>224</v>
+        <v>210</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.35">
@@ -2911,43 +2954,43 @@
         <v>14</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>225</v>
+        <v>211</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>226</v>
+        <v>212</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>227</v>
+        <v>213</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>228</v>
+        <v>292</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>229</v>
+        <v>214</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>230</v>
+        <v>215</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.35">
@@ -2955,43 +2998,43 @@
         <v>15</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>231</v>
+        <v>216</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>232</v>
+        <v>217</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>233</v>
+        <v>218</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>234</v>
+        <v>219</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>235</v>
+        <v>220</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>236</v>
+        <v>221</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>237</v>
+        <v>222</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>275</v>
+        <v>259</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.35">
@@ -2999,43 +3042,43 @@
         <v>16</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>238</v>
+        <v>223</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>239</v>
+        <v>224</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>240</v>
+        <v>225</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>243</v>
+        <v>228</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>244</v>
+        <v>229</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.35">
@@ -3043,43 +3086,43 @@
         <v>17</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>247</v>
+        <v>232</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>32</v>
+        <v>281</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>32</v>
+        <v>282</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>32</v>
+        <v>283</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>248</v>
+        <v>233</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.35">
@@ -3087,43 +3130,43 @@
         <v>18</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>250</v>
+        <v>235</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>32</v>
+        <v>292</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>32</v>
+        <v>284</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>32</v>
+        <v>285</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>252</v>
+        <v>237</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.35">
@@ -3131,43 +3174,43 @@
         <v>19</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>253</v>
+        <v>238</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>254</v>
+        <v>239</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>255</v>
+        <v>240</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>256</v>
+        <v>293</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>257</v>
+        <v>241</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>258</v>
+        <v>242</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>259</v>
+        <v>243</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.35">
@@ -3175,43 +3218,43 @@
         <v>20</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="K23" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="L23" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M23" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>262</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G23" s="3" t="s">
-        <v>263</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I23" s="3" t="s">
-        <v>264</v>
-      </c>
-      <c r="J23" s="3" t="s">
-        <v>265</v>
-      </c>
-      <c r="K23" s="3" t="s">
-        <v>266</v>
-      </c>
-      <c r="L23" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M23" s="2" t="s">
-        <v>276</v>
-      </c>
       <c r="N23" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.35">
@@ -3219,43 +3262,43 @@
         <v>21</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>267</v>
+        <v>251</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>268</v>
+        <v>252</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>269</v>
+        <v>253</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>32</v>
+        <v>288</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>32</v>
+        <v>286</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>32</v>
+        <v>287</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>270</v>
+        <v>254</v>
       </c>
       <c r="L24" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.35">
@@ -3263,43 +3306,43 @@
         <v>22</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>271</v>
+        <v>255</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>272</v>
+        <v>256</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>273</v>
+        <v>257</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>32</v>
+        <v>291</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>32</v>
+        <v>289</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>32</v>
+        <v>290</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>274</v>
+        <v>258</v>
       </c>
       <c r="L25" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>275</v>
+        <v>259</v>
       </c>
       <c r="N25" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>